<commit_message>
Publish MathOntoSpeak research package
</commit_message>
<xml_diff>
--- a/study/analysis/mathontospeak_synthetic_demo_analysis.xlsx
+++ b/study/analysis/mathontospeak_synthetic_demo_analysis.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R26c565d4f3324d80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="2" r:id="Rdc4dd7dbfad04717"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counterbalance" sheetId="3" r:id="Re9e75771b1984074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comprehension Scores" sheetId="4" r:id="R81de29042b6846c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NASA TLX" sheetId="5" r:id="Refa57c2005604abc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCQ Items" sheetId="6" r:id="R5300ce425b8a4a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview Coding" sheetId="7" r:id="R0a3abe2d5a2c4fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demo Provenance" sheetId="8" r:id="R566f88930fea424f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9f7f107121f5467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="2" r:id="R4d42044e22fc4797"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counterbalance" sheetId="3" r:id="R30f2f47b14614328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comprehension Scores" sheetId="4" r:id="R86b2818476194f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NASA TLX" sheetId="5" r:id="Rafa73158617c4724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCQ Items" sheetId="6" r:id="Raf00b1faf92745b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview Coding" sheetId="7" r:id="R7d18ff6ff6e04710"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demo Provenance" sheetId="8" r:id="R851dc114ebfb4a68"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>